<commit_message>
fix: new sample for ensuring run
</commit_message>
<xml_diff>
--- a/tests/sample_data/CCSBT_Global_Catch.xlsx
+++ b/tests/sample_data/CCSBT_Global_Catch.xlsx
@@ -352,7 +352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -384,39 +384,39 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1965</v>
+        <v>1977</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unspecified Surface</t>
+          <t>Longline</t>
         </is>
       </c>
       <c r="E2">
-        <v>6875.99999983391</v>
+        <v>29599.9999895616</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1965</v>
+        <v>1985</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>TW</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -425,21 +425,21 @@
         </is>
       </c>
       <c r="E3">
-        <v>40689.000010831</v>
+        <v>174.000278005</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>1965</v>
+        <v>1994</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ZA</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Korea</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -448,53 +448,398 @@
         </is>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>136.849999968455</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>1966</v>
+        <v>1995</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>??</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Miscellaneous</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Unspecified Surface</t>
+          <t>Longline</t>
         </is>
       </c>
       <c r="E5">
-        <v>8008.00000099823</v>
+        <v>200.71525</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>1966</v>
+        <v>1996</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>NZ</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E6">
+        <v>127.837837391</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>1997</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Korea</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E7">
+        <v>1423.699999998</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>1999</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ZA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E8">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>2001</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E9">
+        <v>85.7859999999998</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>2002</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ZA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E10">
+        <v>17.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>2006</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>JP</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Longline</t>
-        </is>
-      </c>
-      <c r="E6">
-        <v>39643.9999869011</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E11">
+        <v>4207.00000087317</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>2007</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PH</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E12">
+        <v>45.9195</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>2010</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E13">
+        <v>1208.000000005</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>2012</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E14">
+        <v>58.1715518836568</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>2015</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NZ</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E15">
+        <v>922.189662572</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>2018</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Purse Seine</t>
+        </is>
+      </c>
+      <c r="E16">
+        <v>5366.63925645472</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>2018</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Korea</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E17">
+        <v>1268.428260001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>2019</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E18">
+        <v>1228.999999997</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>2020</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E19">
+        <v>5928.99999810466</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>2022</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="E20">
+        <v>5886.99999811205</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>2024</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pole and Line</t>
+        </is>
+      </c>
+      <c r="E21">
+        <v>1.133752</v>
       </c>
     </row>
   </sheetData>
@@ -504,7 +849,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -541,16 +886,16 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1965</v>
+        <v>1967</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -560,44 +905,44 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unspecified Surface</t>
+          <t>Longline</t>
         </is>
       </c>
       <c r="F2">
-        <v>4675.02456514981</v>
+        <v>50474.5483295708</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1965</v>
+        <v>1971</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Indian</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Unspecified Surface</t>
+          <t>Longline</t>
         </is>
       </c>
       <c r="F3">
-        <v>2200.9754346841</v>
+        <v>23137.560073553</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>1965</v>
+        <v>1977</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -620,12 +965,12 @@
         </is>
       </c>
       <c r="F4">
-        <v>15.3320115866524</v>
+        <v>4462.51053480109</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>1965</v>
+        <v>1980</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -639,7 +984,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Indian</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -648,35 +993,455 @@
         </is>
       </c>
       <c r="F5">
-        <v>28094.6361130015</v>
+        <v>3085.99132069364</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>1965</v>
+        <v>1983</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>??</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Miscellaneous</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F6">
+        <v>7.12876</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>1984</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F7">
+        <v>243.404997567</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>1995</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F8">
+        <v>828.96989</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>1997</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F9">
+        <v>782.911591338</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>2005</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Korea</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F10">
+        <v>37.95</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>2006</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>JP</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F11">
+        <v>3444.90711517148</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>2006</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Korea</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Atlantic</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F12">
+        <v>0.594120444</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>2009</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Research and Other</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Troll</t>
+        </is>
+      </c>
+      <c r="F13">
+        <v>0.2143</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>2010</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>NZ</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>Pacific</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Longline</t>
-        </is>
-      </c>
-      <c r="F6">
-        <v>12579.0318862428</v>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Troll</t>
+        </is>
+      </c>
+      <c r="F14">
+        <v>0.100974159</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>2010</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ZA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F15">
+        <v>7.75005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>2014</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Purse Seine</t>
+        </is>
+      </c>
+      <c r="F16">
+        <v>4168.08605626565</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>2014</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>NZ</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pacific</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F17">
+        <v>824.341797768</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>2017</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Korea</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F18">
+        <v>29.383682664</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>2018</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NZ</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Pacific</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F19">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>2023</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Korea</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F20">
+        <v>148.566536132</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>2024</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Longline</t>
+        </is>
+      </c>
+      <c r="F21">
+        <v>1224.3765</v>
       </c>
     </row>
   </sheetData>

</xml_diff>